<commit_message>
content: align VALCAN pack with current V2 extractor
</commit_message>
<xml_diff>
--- a/data/canary/valcan_pack_2026-04-12/_VALCAN_2026/00_README/valcanary_ground_truth_index.xlsx
+++ b/data/canary/valcan_pack_2026-04-12/_VALCAN_2026/00_README/valcanary_ground_truth_index.xlsx
@@ -632,7 +632,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>5 distinct parts failed during 4 lightning-related service events across 3 validation sites: VALSITE-ALPHA, VALSITE-BRAVO, and VALSITE-CHARLIE.</t>
+          <t>5 distinct parts failed during 4 lightning-related service events across 3 validation sites: Validation Alpha Site, Validation Bravo Site, and Validation Charlie Site.</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -835,7 +835,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Validation shipments to VALSITE-ALPHA</t>
+          <t>Validation shipments to Validation Alpha Site</t>
         </is>
       </c>
       <c r="B8" t="n">

</xml_diff>